<commit_message>
Restore Region-Wise KPIs, classify DZL shoes gender by size without Unisex, and eliminate zero values
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="315" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="91">
   <si>
     <t>Brand</t>
   </si>
@@ -88,18 +88,15 @@
     <t>360 degree cleaning brush</t>
   </si>
   <si>
+    <t>KIDS Socks</t>
+  </si>
+  <si>
     <t>WOMANS Boat Socks</t>
   </si>
   <si>
-    <t>KIDS Socks</t>
-  </si>
-  <si>
     <t>MANS Boat Socks 3 pairs</t>
   </si>
   <si>
-    <t>Household Utensils</t>
-  </si>
-  <si>
     <t>Foam Insole</t>
   </si>
   <si>
@@ -115,39 +112,30 @@
     <t>MANS No-show Socks</t>
   </si>
   <si>
+    <t>CL Roam Hands Free Traine</t>
+  </si>
+  <si>
     <t>low rise wOMANS socks 3 p</t>
   </si>
   <si>
     <t>WOMANS Low-cut Socks</t>
   </si>
   <si>
-    <t>CL Roam Hands Free Traine</t>
-  </si>
-  <si>
-    <t>DZL-Shoe Deodorization Bo</t>
-  </si>
-  <si>
     <t>6971340016867</t>
   </si>
   <si>
+    <t>6957352843639</t>
+  </si>
+  <si>
     <t>6957352859289</t>
   </si>
   <si>
-    <t>6957352843639</t>
-  </si>
-  <si>
     <t>6957352859265</t>
   </si>
   <si>
     <t>6957352859357</t>
   </si>
   <si>
-    <t>6957352859661</t>
-  </si>
-  <si>
-    <t>6957352859678</t>
-  </si>
-  <si>
     <t>6957352875425</t>
   </si>
   <si>
@@ -172,6 +160,12 @@
     <t>6957352803244</t>
   </si>
   <si>
+    <t>DS0771040840</t>
+  </si>
+  <si>
+    <t>6957352843691</t>
+  </si>
+  <si>
     <t>6957352859258</t>
   </si>
   <si>
@@ -181,39 +175,24 @@
     <t>6957352789913</t>
   </si>
   <si>
-    <t>6957352843691</t>
-  </si>
-  <si>
-    <t>DS0771040840</t>
-  </si>
-  <si>
-    <t>6957352858961</t>
-  </si>
-  <si>
     <t>6957352859333</t>
   </si>
   <si>
     <t>720976</t>
   </si>
   <si>
+    <t>720922</t>
+  </si>
+  <si>
     <t>720944</t>
   </si>
   <si>
-    <t>720922</t>
-  </si>
-  <si>
     <t>720951</t>
   </si>
   <si>
     <t>720933</t>
   </si>
   <si>
-    <t>720966</t>
-  </si>
-  <si>
-    <t>720960</t>
-  </si>
-  <si>
     <t>731029</t>
   </si>
   <si>
@@ -238,6 +217,12 @@
     <t>720868</t>
   </si>
   <si>
+    <t>726186</t>
+  </si>
+  <si>
+    <t>720918</t>
+  </si>
+  <si>
     <t>730709</t>
   </si>
   <si>
@@ -247,36 +232,21 @@
     <t>720808</t>
   </si>
   <si>
-    <t>720918</t>
-  </si>
-  <si>
-    <t>726186</t>
-  </si>
-  <si>
-    <t>730692</t>
-  </si>
-  <si>
     <t>720935</t>
   </si>
   <si>
     <t xml:space="preserve">360 degree cleaning brush UNISEX 0 </t>
   </si>
   <si>
+    <t>DZL Childrens Low-cut Socks # 16-18</t>
+  </si>
+  <si>
     <t>DZL-5A Antibacterial and Anti pilli</t>
   </si>
   <si>
-    <t>DZL Childrens Low-cut Socks # 16-18</t>
-  </si>
-  <si>
     <t>DZL-5A Antibacterial Foot Loop Wome</t>
   </si>
   <si>
-    <t>DZL-Vacuum Cup # green -600ML</t>
-  </si>
-  <si>
-    <t>DZL-Vacuum Cup # white -600ML</t>
-  </si>
-  <si>
     <t>Foam Insole UNISEX Beige Accessorie</t>
   </si>
   <si>
@@ -292,6 +262,12 @@
     <t>DZL Mens No-show Socks-Black#2015</t>
   </si>
   <si>
+    <t>CL Roam Hands Free Trainer MAN Blac</t>
+  </si>
+  <si>
+    <t>DZL Childrens Low-cut Socks # 18-20</t>
+  </si>
+  <si>
     <t>DZL-5A antibacterial and anti pilli</t>
   </si>
   <si>
@@ -301,19 +277,10 @@
     <t>DZL Ladys Low-cut Socks-Black</t>
   </si>
   <si>
-    <t>DZL Childrens Low-cut Socks # 18-20</t>
-  </si>
-  <si>
-    <t>CL Roam Hands Free Trainer MAN Blac</t>
-  </si>
-  <si>
-    <t>DZL-Shoe Deodorization Box UNISEX O</t>
-  </si>
-  <si>
     <t>Accessories</t>
   </si>
   <si>
-    <t>Footwear (Shoes)</t>
+    <t>Shoes</t>
   </si>
   <si>
     <t>Central Warehouse (KSWH - Limited: 1)</t>
@@ -651,7 +618,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O31"/>
+  <dimension ref="A1:O28"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -718,16 +685,16 @@
         <v>23</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H2" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="I2" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -745,7 +712,7 @@
         <v>19</v>
       </c>
       <c r="O2" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -765,16 +732,16 @@
         <v>24</v>
       </c>
       <c r="F3" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="H3" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="I3" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -792,7 +759,7 @@
         <v>9</v>
       </c>
       <c r="O3" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -812,16 +779,16 @@
         <v>25</v>
       </c>
       <c r="F4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="H4" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="I4" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -839,7 +806,7 @@
         <v>9</v>
       </c>
       <c r="O4" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -859,16 +826,16 @@
         <v>26</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H5" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -886,7 +853,7 @@
         <v>8</v>
       </c>
       <c r="O5" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -906,16 +873,16 @@
         <v>26</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="H6" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="I6" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -933,7 +900,7 @@
         <v>8</v>
       </c>
       <c r="O6" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -950,19 +917,19 @@
         <v>21</v>
       </c>
       <c r="E7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="H7" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="I7" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -980,7 +947,7 @@
         <v>7</v>
       </c>
       <c r="O7" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -991,25 +958,25 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D8" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E8" t="s">
         <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="G8" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="I8" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -1024,10 +991,10 @@
         <v>3</v>
       </c>
       <c r="N8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="O8" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -1044,19 +1011,19 @@
         <v>20</v>
       </c>
       <c r="E9" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G9" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="H9" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="I9" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -1074,7 +1041,7 @@
         <v>6</v>
       </c>
       <c r="O9" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -1091,19 +1058,19 @@
         <v>20</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F10" t="s">
         <v>41</v>
       </c>
       <c r="G10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H10" t="s">
-        <v>84</v>
+        <v>75</v>
       </c>
       <c r="I10" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1112,16 +1079,16 @@
         <v>1</v>
       </c>
       <c r="L10">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="M10">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N10">
         <v>6</v>
       </c>
       <c r="O10" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1132,25 +1099,25 @@
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s">
         <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G11" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="H11" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="I11" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -1159,16 +1126,16 @@
         <v>1</v>
       </c>
       <c r="L11">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="M11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="N11">
         <v>6</v>
       </c>
       <c r="O11" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1185,19 +1152,19 @@
         <v>20</v>
       </c>
       <c r="E12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G12" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="H12" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="I12" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1215,7 +1182,7 @@
         <v>6</v>
       </c>
       <c r="O12" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1226,25 +1193,25 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G13" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="H13" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="I13" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -1256,13 +1223,13 @@
         <v>0.2</v>
       </c>
       <c r="M13">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N13">
         <v>6</v>
       </c>
       <c r="O13" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -1279,19 +1246,19 @@
         <v>20</v>
       </c>
       <c r="E14" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F14" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H14" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="I14" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -1303,13 +1270,13 @@
         <v>0.2</v>
       </c>
       <c r="M14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="N14">
         <v>6</v>
       </c>
       <c r="O14" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -1326,19 +1293,19 @@
         <v>22</v>
       </c>
       <c r="E15" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F15" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="G15" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="H15" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="I15" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -1356,7 +1323,7 @@
         <v>6</v>
       </c>
       <c r="O15" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -1373,19 +1340,19 @@
         <v>22</v>
       </c>
       <c r="E16" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="H16" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="I16" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -1403,7 +1370,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -1414,25 +1381,25 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D17" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E17" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F17" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="G17" t="s">
-        <v>68</v>
+        <v>56</v>
       </c>
       <c r="H17" t="s">
-        <v>88</v>
+        <v>75</v>
       </c>
       <c r="I17" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -1450,7 +1417,7 @@
         <v>6</v>
       </c>
       <c r="O17" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -1467,19 +1434,19 @@
         <v>21</v>
       </c>
       <c r="E18" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="F18" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H18" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="I18" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -1491,13 +1458,13 @@
         <v>0.2</v>
       </c>
       <c r="M18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N18">
         <v>6</v>
       </c>
       <c r="O18" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1508,43 +1475,43 @@
         <v>16</v>
       </c>
       <c r="C19" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D19" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E19" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F19" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G19" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="H19" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="I19" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J19">
         <v>1</v>
       </c>
       <c r="K19">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L19">
         <v>0.2</v>
       </c>
       <c r="M19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N19">
         <v>6</v>
       </c>
       <c r="O19" t="s">
-        <v>100</v>
+        <v>90</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1555,25 +1522,25 @@
         <v>16</v>
       </c>
       <c r="C20" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D20" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E20" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="F20" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="G20" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="H20" t="s">
         <v>82</v>
       </c>
       <c r="I20" t="s">
-        <v>98</v>
+        <v>88</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -1591,7 +1558,7 @@
         <v>6</v>
       </c>
       <c r="O20" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -1602,31 +1569,31 @@
         <v>16</v>
       </c>
       <c r="C21" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E21" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="F21" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="G21" t="s">
+        <v>54</v>
+      </c>
+      <c r="H21" t="s">
         <v>73</v>
       </c>
-      <c r="H21" t="s">
-        <v>91</v>
-      </c>
       <c r="I21" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J21">
         <v>1</v>
       </c>
       <c r="K21">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L21">
         <v>0.2</v>
@@ -1638,7 +1605,7 @@
         <v>6</v>
       </c>
       <c r="O21" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -1649,25 +1616,25 @@
         <v>16</v>
       </c>
       <c r="C22" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D22" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E22" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="F22" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="H22" t="s">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="I22" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -1685,7 +1652,7 @@
         <v>6</v>
       </c>
       <c r="O22" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -1702,19 +1669,19 @@
         <v>20</v>
       </c>
       <c r="E23" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="F23" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="G23" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="H23" t="s">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="I23" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -1732,7 +1699,7 @@
         <v>6</v>
       </c>
       <c r="O23" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -1749,19 +1716,19 @@
         <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F24" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G24" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="H24" t="s">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="I24" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -1779,7 +1746,7 @@
         <v>6</v>
       </c>
       <c r="O24" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -1790,25 +1757,25 @@
         <v>16</v>
       </c>
       <c r="C25" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D25" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="F25" t="s">
-        <v>37</v>
+        <v>52</v>
       </c>
       <c r="G25" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="H25" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="I25" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -1826,7 +1793,7 @@
         <v>6</v>
       </c>
       <c r="O25" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -1837,25 +1804,25 @@
         <v>16</v>
       </c>
       <c r="C26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E26" t="s">
         <v>25</v>
       </c>
       <c r="F26" t="s">
-        <v>55</v>
+        <v>43</v>
       </c>
       <c r="G26" t="s">
-        <v>77</v>
+        <v>62</v>
       </c>
       <c r="H26" t="s">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="I26" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -1864,16 +1831,16 @@
         <v>1</v>
       </c>
       <c r="L26">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="M26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N26">
         <v>6</v>
       </c>
       <c r="O26" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -1884,25 +1851,25 @@
         <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E27" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F27" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G27" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="H27" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="I27" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -1920,7 +1887,7 @@
         <v>6</v>
       </c>
       <c r="O27" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -1931,25 +1898,25 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E28" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="F28" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="G28" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="H28" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="I28" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="J28">
         <v>1</v>
@@ -1967,148 +1934,7 @@
         <v>6</v>
       </c>
       <c r="O28" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="29" spans="1:15">
-      <c r="A29" t="s">
-        <v>15</v>
-      </c>
-      <c r="B29" t="s">
-        <v>16</v>
-      </c>
-      <c r="C29" t="s">
-        <v>19</v>
-      </c>
-      <c r="D29" t="s">
-        <v>22</v>
-      </c>
-      <c r="E29" t="s">
-        <v>35</v>
-      </c>
-      <c r="F29" t="s">
-        <v>56</v>
-      </c>
-      <c r="G29" t="s">
-        <v>78</v>
-      </c>
-      <c r="H29" t="s">
-        <v>96</v>
-      </c>
-      <c r="I29" t="s">
-        <v>99</v>
-      </c>
-      <c r="J29">
-        <v>1</v>
-      </c>
-      <c r="K29">
-        <v>1</v>
-      </c>
-      <c r="L29">
-        <v>0.1</v>
-      </c>
-      <c r="M29">
-        <v>7</v>
-      </c>
-      <c r="N29">
-        <v>6</v>
-      </c>
-      <c r="O29" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="30" spans="1:15">
-      <c r="A30" t="s">
-        <v>15</v>
-      </c>
-      <c r="B30" t="s">
-        <v>16</v>
-      </c>
-      <c r="C30" t="s">
-        <v>17</v>
-      </c>
-      <c r="D30" t="s">
-        <v>20</v>
-      </c>
-      <c r="E30" t="s">
-        <v>36</v>
-      </c>
-      <c r="F30" t="s">
-        <v>57</v>
-      </c>
-      <c r="G30" t="s">
-        <v>79</v>
-      </c>
-      <c r="H30" t="s">
-        <v>97</v>
-      </c>
-      <c r="I30" t="s">
-        <v>98</v>
-      </c>
-      <c r="J30">
-        <v>1</v>
-      </c>
-      <c r="K30">
-        <v>1</v>
-      </c>
-      <c r="L30">
-        <v>0.1</v>
-      </c>
-      <c r="M30">
-        <v>7</v>
-      </c>
-      <c r="N30">
-        <v>6</v>
-      </c>
-      <c r="O30" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="31" spans="1:15">
-      <c r="A31" t="s">
-        <v>15</v>
-      </c>
-      <c r="B31" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" t="s">
-        <v>17</v>
-      </c>
-      <c r="D31" t="s">
-        <v>20</v>
-      </c>
-      <c r="E31" t="s">
-        <v>26</v>
-      </c>
-      <c r="F31" t="s">
-        <v>58</v>
-      </c>
-      <c r="G31" t="s">
-        <v>80</v>
-      </c>
-      <c r="H31" t="s">
-        <v>90</v>
-      </c>
-      <c r="I31" t="s">
-        <v>98</v>
-      </c>
-      <c r="J31">
-        <v>1</v>
-      </c>
-      <c r="K31">
-        <v>1</v>
-      </c>
-      <c r="L31">
-        <v>0.1</v>
-      </c>
-      <c r="M31">
-        <v>7</v>
-      </c>
-      <c r="N31">
-        <v>6</v>
-      </c>
-      <c r="O31" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix repl_rows_html NameError, remove telegram completely, isolate DZL regions and enable drilldowns
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="285" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="94">
   <si>
     <t>Brand</t>
   </si>
@@ -139,15 +139,15 @@
     <t>6957352875425</t>
   </si>
   <si>
+    <t>6957352859036</t>
+  </si>
+  <si>
+    <t>6957352859340</t>
+  </si>
+  <si>
     <t>6957352859272</t>
   </si>
   <si>
-    <t>6957352859036</t>
-  </si>
-  <si>
-    <t>6957352859340</t>
-  </si>
-  <si>
     <t>6971277830871</t>
   </si>
   <si>
@@ -166,6 +166,9 @@
     <t>6957352843691</t>
   </si>
   <si>
+    <t>6957352859333</t>
+  </si>
+  <si>
     <t>6957352859258</t>
   </si>
   <si>
@@ -175,7 +178,7 @@
     <t>6957352789913</t>
   </si>
   <si>
-    <t>6957352859333</t>
+    <t>6957352875371</t>
   </si>
   <si>
     <t>720976</t>
@@ -196,15 +199,15 @@
     <t>731029</t>
   </si>
   <si>
+    <t>720939</t>
+  </si>
+  <si>
+    <t>720957</t>
+  </si>
+  <si>
     <t>720953</t>
   </si>
   <si>
-    <t>720939</t>
-  </si>
-  <si>
-    <t>720957</t>
-  </si>
-  <si>
     <t>720978</t>
   </si>
   <si>
@@ -223,6 +226,9 @@
     <t>720918</t>
   </si>
   <si>
+    <t>720935</t>
+  </si>
+  <si>
     <t>730709</t>
   </si>
   <si>
@@ -232,7 +238,7 @@
     <t>720808</t>
   </si>
   <si>
-    <t>720935</t>
+    <t>731017</t>
   </si>
   <si>
     <t xml:space="preserve">360 degree cleaning brush UNISEX 0 </t>
@@ -275,6 +281,9 @@
   </si>
   <si>
     <t>DZL Ladys Low-cut Socks-Black</t>
+  </si>
+  <si>
+    <t>Foam Insole UNISEX Black Accessorie</t>
   </si>
   <si>
     <t>Accessories</t>
@@ -618,7 +627,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O28"/>
+  <dimension ref="A1:O29"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:15">
@@ -688,13 +697,13 @@
         <v>35</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H2" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -703,16 +712,16 @@
         <v>1</v>
       </c>
       <c r="L2">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="M2">
         <v>1</v>
       </c>
       <c r="N2">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="O2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:15">
@@ -735,13 +744,13 @@
         <v>36</v>
       </c>
       <c r="G3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H3" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="I3" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -759,7 +768,7 @@
         <v>9</v>
       </c>
       <c r="O3" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:15">
@@ -782,13 +791,13 @@
         <v>37</v>
       </c>
       <c r="G4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="H4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -806,7 +815,7 @@
         <v>9</v>
       </c>
       <c r="O4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:15">
@@ -817,10 +826,10 @@
         <v>16</v>
       </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E5" t="s">
         <v>26</v>
@@ -829,13 +838,13 @@
         <v>38</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I5" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -853,7 +862,7 @@
         <v>8</v>
       </c>
       <c r="O5" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:15">
@@ -864,10 +873,10 @@
         <v>16</v>
       </c>
       <c r="C6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s">
         <v>26</v>
@@ -876,13 +885,13 @@
         <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I6" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -900,7 +909,7 @@
         <v>8</v>
       </c>
       <c r="O6" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" spans="1:15">
@@ -923,13 +932,13 @@
         <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H7" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="I7" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -947,7 +956,7 @@
         <v>7</v>
       </c>
       <c r="O7" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:15">
@@ -958,25 +967,25 @@
         <v>16</v>
       </c>
       <c r="C8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E8" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G8" t="s">
         <v>59</v>
       </c>
       <c r="H8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I8" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -994,7 +1003,7 @@
         <v>6</v>
       </c>
       <c r="O8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:15">
@@ -1005,25 +1014,25 @@
         <v>16</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -1041,7 +1050,7 @@
         <v>6</v>
       </c>
       <c r="O9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:15">
@@ -1052,25 +1061,25 @@
         <v>16</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F10" t="s">
         <v>41</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H10" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I10" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -1088,7 +1097,7 @@
         <v>6</v>
       </c>
       <c r="O10" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:15">
@@ -1099,25 +1108,25 @@
         <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E11" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s">
         <v>42</v>
       </c>
       <c r="G11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H11" t="s">
         <v>78</v>
       </c>
       <c r="I11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -1135,7 +1144,7 @@
         <v>6</v>
       </c>
       <c r="O11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="12" spans="1:15">
@@ -1152,19 +1161,19 @@
         <v>20</v>
       </c>
       <c r="E12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F12" t="s">
         <v>43</v>
       </c>
       <c r="G12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H12" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="I12" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -1182,7 +1191,7 @@
         <v>6</v>
       </c>
       <c r="O12" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="13" spans="1:15">
@@ -1193,25 +1202,25 @@
         <v>16</v>
       </c>
       <c r="C13" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G13" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H13" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="I13" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -1223,13 +1232,13 @@
         <v>0.2</v>
       </c>
       <c r="M13">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N13">
         <v>6</v>
       </c>
       <c r="O13" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="14" spans="1:15">
@@ -1240,25 +1249,25 @@
         <v>16</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D14" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="G14" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="H14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I14" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -1276,7 +1285,7 @@
         <v>6</v>
       </c>
       <c r="O14" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="15" spans="1:15">
@@ -1299,13 +1308,13 @@
         <v>45</v>
       </c>
       <c r="G15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="I15" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -1323,7 +1332,7 @@
         <v>6</v>
       </c>
       <c r="O15" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:15">
@@ -1334,10 +1343,10 @@
         <v>16</v>
       </c>
       <c r="C16" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D16" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s">
         <v>29</v>
@@ -1346,13 +1355,13 @@
         <v>44</v>
       </c>
       <c r="G16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H16" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I16" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -1370,7 +1379,7 @@
         <v>6</v>
       </c>
       <c r="O16" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:15">
@@ -1381,25 +1390,25 @@
         <v>16</v>
       </c>
       <c r="C17" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E17" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F17" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="G17" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="H17" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="I17" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J17">
         <v>1</v>
@@ -1417,7 +1426,7 @@
         <v>6</v>
       </c>
       <c r="O17" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:15">
@@ -1440,13 +1449,13 @@
         <v>46</v>
       </c>
       <c r="G18" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H18" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I18" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J18">
         <v>1</v>
@@ -1464,7 +1473,7 @@
         <v>6</v>
       </c>
       <c r="O18" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" spans="1:15">
@@ -1487,13 +1496,13 @@
         <v>47</v>
       </c>
       <c r="G19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="I19" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J19">
         <v>1</v>
@@ -1511,7 +1520,7 @@
         <v>6</v>
       </c>
       <c r="O19" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="20" spans="1:15">
@@ -1534,13 +1543,13 @@
         <v>48</v>
       </c>
       <c r="G20" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H20" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="I20" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="J20">
         <v>1</v>
@@ -1558,7 +1567,7 @@
         <v>6</v>
       </c>
       <c r="O20" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:15">
@@ -1581,13 +1590,13 @@
         <v>35</v>
       </c>
       <c r="G21" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H21" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="I21" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J21">
         <v>1</v>
@@ -1605,7 +1614,7 @@
         <v>6</v>
       </c>
       <c r="O21" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:15">
@@ -1628,13 +1637,13 @@
         <v>49</v>
       </c>
       <c r="G22" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H22" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I22" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J22">
         <v>1</v>
@@ -1652,7 +1661,7 @@
         <v>6</v>
       </c>
       <c r="O22" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="1:15">
@@ -1669,19 +1678,19 @@
         <v>20</v>
       </c>
       <c r="E23" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="F23" t="s">
         <v>50</v>
       </c>
       <c r="G23" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H23" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="I23" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J23">
         <v>1</v>
@@ -1699,7 +1708,7 @@
         <v>6</v>
       </c>
       <c r="O23" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="24" spans="1:15">
@@ -1716,19 +1725,19 @@
         <v>20</v>
       </c>
       <c r="E24" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="F24" t="s">
         <v>51</v>
       </c>
       <c r="G24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H24" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="I24" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J24">
         <v>1</v>
@@ -1746,7 +1755,7 @@
         <v>6</v>
       </c>
       <c r="O24" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="25" spans="1:15">
@@ -1763,19 +1772,19 @@
         <v>20</v>
       </c>
       <c r="E25" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="F25" t="s">
         <v>52</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H25" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I25" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J25">
         <v>1</v>
@@ -1793,7 +1802,7 @@
         <v>6</v>
       </c>
       <c r="O25" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:15">
@@ -1804,25 +1813,25 @@
         <v>16</v>
       </c>
       <c r="C26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D26" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E26" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="F26" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="G26" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="H26" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="I26" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J26">
         <v>1</v>
@@ -1831,16 +1840,16 @@
         <v>1</v>
       </c>
       <c r="L26">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M26">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="N26">
         <v>6</v>
       </c>
       <c r="O26" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="27" spans="1:15">
@@ -1851,25 +1860,25 @@
         <v>16</v>
       </c>
       <c r="C27" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D27" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E27" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F27" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="G27" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="H27" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="I27" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J27">
         <v>1</v>
@@ -1887,7 +1896,7 @@
         <v>6</v>
       </c>
       <c r="O27" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="28" spans="1:15">
@@ -1898,25 +1907,25 @@
         <v>16</v>
       </c>
       <c r="C28" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D28" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E28" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F28" t="s">
-        <v>53</v>
+        <v>41</v>
       </c>
       <c r="G28" t="s">
-        <v>72</v>
+        <v>61</v>
       </c>
       <c r="H28" t="s">
         <v>80</v>
       </c>
       <c r="I28" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="J28">
         <v>1</v>
@@ -1934,7 +1943,54 @@
         <v>6</v>
       </c>
       <c r="O28" t="s">
-        <v>89</v>
+        <v>92</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15">
+      <c r="A29" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" t="s">
+        <v>21</v>
+      </c>
+      <c r="E29" t="s">
+        <v>25</v>
+      </c>
+      <c r="F29" t="s">
+        <v>42</v>
+      </c>
+      <c r="G29" t="s">
+        <v>62</v>
+      </c>
+      <c r="H29" t="s">
+        <v>78</v>
+      </c>
+      <c r="I29" t="s">
+        <v>90</v>
+      </c>
+      <c r="J29">
+        <v>1</v>
+      </c>
+      <c r="K29">
+        <v>1</v>
+      </c>
+      <c r="L29">
+        <v>0.1</v>
+      </c>
+      <c r="M29">
+        <v>7</v>
+      </c>
+      <c r="N29">
+        <v>6</v>
+      </c>
+      <c r="O29" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix replenishment recommendations to prioritize shoes, handle zero warehouse stock with IST routing, and resolve python variable definitions
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -73,7 +73,7 @@
     <t>2 - Routine (Accessory)</t>
   </si>
   <si>
-    <t>Predictive WH Replenishment</t>
+    <t>Store Transfer (IST - Peer Network)</t>
   </si>
   <si>
     <t>K111</t>
@@ -856,10 +856,10 @@
     <t>⚠️ Stock-Out in 7d (Vel: 0.1/d)</t>
   </si>
   <si>
-    <t>Central Warehouse (KSWH - Limited: 1)</t>
-  </si>
-  <si>
-    <t>Central Warehouse (KSWH - Limited: 0)</t>
+    <t>Peer Store Network (WH Stock: 1 - Cross-Store Balance)</t>
+  </si>
+  <si>
+    <t>Peer Store Network (WH Stock: 0 - Cross-Store Balance)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fix business charts rendering, implement complete drilldown table, and ensure IST routing when WH stock is zero
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -73,7 +73,7 @@
     <t>2 - Routine (Accessory)</t>
   </si>
   <si>
-    <t>Store Transfer (IST - Peer Network)</t>
+    <t>Predictive WH Replenishment</t>
   </si>
   <si>
     <t>K111</t>
@@ -856,10 +856,10 @@
     <t>⚠️ Stock-Out in 7d (Vel: 0.1/d)</t>
   </si>
   <si>
-    <t>Peer Store Network (WH Stock: 1 - Cross-Store Balance)</t>
-  </si>
-  <si>
-    <t>Peer Store Network (WH Stock: 0 - Cross-Store Balance)</t>
+    <t>Central Warehouse (KSWH - Limited: 1)</t>
+  </si>
+  <si>
+    <t>Central Warehouse (KSWH - Limited: 0)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fix business charts DOM rendering, add store-wise Top/Low 20 shoes filter, and ensure robust IST routing
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -73,7 +73,7 @@
     <t>2 - Routine (Accessory)</t>
   </si>
   <si>
-    <t>Predictive WH Replenishment</t>
+    <t>Store Transfer (IST - Peer Network)</t>
   </si>
   <si>
     <t>K111</t>
@@ -856,10 +856,10 @@
     <t>⚠️ Stock-Out in 7d (Vel: 0.1/d)</t>
   </si>
   <si>
-    <t>Central Warehouse (KSWH - Limited: 1)</t>
-  </si>
-  <si>
-    <t>Central Warehouse (KSWH - Limited: 0)</t>
+    <t>Peer Store Network (WH Stock: 1 - Cross-Store Balance)</t>
+  </si>
+  <si>
+    <t>Peer Store Network (WH Stock: 0 - Cross-Store Balance)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fix top_cats_str key error, repair business charts rendering, and add store-wise top/low 20 shoes filter with IST routing
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -73,7 +73,7 @@
     <t>2 - Routine (Accessory)</t>
   </si>
   <si>
-    <t>Store Transfer (IST - Peer Network)</t>
+    <t>Store Transfer (IST - Network Balancing)</t>
   </si>
   <si>
     <t>K111</t>
@@ -856,10 +856,10 @@
     <t>⚠️ Stock-Out in 7d (Vel: 0.1/d)</t>
   </si>
   <si>
-    <t>Peer Store Network (WH Stock: 1 - Cross-Store Balance)</t>
-  </si>
-  <si>
-    <t>Peer Store Network (WH Stock: 0 - Cross-Store Balance)</t>
+    <t>Peer Store Network (WH Stock: 1 - Cross-Store Balancing)</t>
+  </si>
+  <si>
+    <t>Peer Store Network (WH Stock: 0 - Cross-Store Balancing)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Fix syntax error unmatched parenthesis on line 178
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="72">
   <si>
     <t>Brand</t>
   </si>
@@ -40,9 +40,42 @@
     <t>DZL</t>
   </si>
   <si>
+    <t>DZL Riyadh U-Walk</t>
+  </si>
+  <si>
     <t>DZL Riyadh Park</t>
   </si>
   <si>
+    <t>725536</t>
+  </si>
+  <si>
+    <t>725570</t>
+  </si>
+  <si>
+    <t>725678</t>
+  </si>
+  <si>
+    <t>725879</t>
+  </si>
+  <si>
+    <t>726672</t>
+  </si>
+  <si>
+    <t>730127</t>
+  </si>
+  <si>
+    <t>794027</t>
+  </si>
+  <si>
+    <t>794041</t>
+  </si>
+  <si>
+    <t>800131</t>
+  </si>
+  <si>
+    <t>810013</t>
+  </si>
+  <si>
     <t>720969</t>
   </si>
   <si>
@@ -103,19 +136,34 @@
     <t>726806</t>
   </si>
   <si>
-    <t>729571</t>
-  </si>
-  <si>
-    <t>794015</t>
-  </si>
-  <si>
-    <t>794016</t>
-  </si>
-  <si>
-    <t>794018</t>
-  </si>
-  <si>
-    <t>794020</t>
+    <t>CL Wander Trainer MAN White 40</t>
+  </si>
+  <si>
+    <t>CL Wander Trainer WOMAN White 38</t>
+  </si>
+  <si>
+    <t>CL Highland Sock Trainer WOMAN White 38</t>
+  </si>
+  <si>
+    <t>CL Canyon Wool Trainer PS Fog Grey/Light Grey 26</t>
+  </si>
+  <si>
+    <t>BR Ripple Nylon Runner Sneaker MAN Black/Dark Grey 41</t>
+  </si>
+  <si>
+    <t>AQ Three-Strap SS Sandal WOMAN Cocoa 38</t>
+  </si>
+  <si>
+    <t>BR-Nexus-Knit-Runner-Sneaker-MAN-Black-44</t>
+  </si>
+  <si>
+    <t>BR-Nexus-Knit-Runner-Sneaker-MAN-Black-43</t>
+  </si>
+  <si>
+    <t>CL Ripple Wool TrainerCreamMEN</t>
+  </si>
+  <si>
+    <t>CL WANDER TRAINER WOMAN WHITE 36.5</t>
   </si>
   <si>
     <t>DZL-SHOE DEODORIZER SPRAY#150ML UNISEX 0 Care Products0UNISEX</t>
@@ -178,22 +226,7 @@
     <t>CL Classic SS Trainer KIDS Black 26</t>
   </si>
   <si>
-    <t>BR Ripple Runner Sneaker MAN Black/Grey 40</t>
-  </si>
-  <si>
-    <t>BR-Nexus-Knit-Runner-Sneaker-MAN-Black-40</t>
-  </si>
-  <si>
-    <t>BR-Nexus-Knit-Runner-Sneaker-MAN-Pale-Beige-45</t>
-  </si>
-  <si>
-    <t>BR-Nexus-Knit-Runner-Sneaker-MAN-Pale-Beige-41</t>
-  </si>
-  <si>
-    <t>BR-Nexus-Knit-Runner-Sneaker-MAN-Pale-Beige-44</t>
-  </si>
-  <si>
-    <t>DZL Riyadh U-Walk</t>
+    <t>DZL Solitaire</t>
   </si>
   <si>
     <t>🏙️ Same City</t>
@@ -528,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -562,19 +595,19 @@
         <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F2">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="G2" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -585,19 +618,19 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D3" t="s">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G3" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -608,19 +641,19 @@
         <v>8</v>
       </c>
       <c r="C4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G4" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -631,19 +664,19 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F5">
         <v>2</v>
       </c>
       <c r="G5" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:7">
@@ -654,19 +687,19 @@
         <v>8</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:7">
@@ -677,19 +710,19 @@
         <v>8</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D7" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -700,19 +733,19 @@
         <v>8</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D8" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F8">
         <v>2</v>
       </c>
       <c r="G8" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -723,19 +756,19 @@
         <v>8</v>
       </c>
       <c r="C9" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F9">
         <v>2</v>
       </c>
       <c r="G9" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -746,19 +779,19 @@
         <v>8</v>
       </c>
       <c r="C10" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F10">
         <v>2</v>
       </c>
       <c r="G10" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -769,19 +802,19 @@
         <v>8</v>
       </c>
       <c r="C11" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F11">
         <v>2</v>
       </c>
       <c r="G11" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -789,22 +822,22 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C12" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D12" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F12">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="G12" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -812,22 +845,22 @@
         <v>7</v>
       </c>
       <c r="B13" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D13" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E13" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F13">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G13" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -835,22 +868,22 @@
         <v>7</v>
       </c>
       <c r="B14" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C14" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D14" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="E14" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F14">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G14" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -858,22 +891,22 @@
         <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D15" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="E15" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F15">
         <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -881,22 +914,22 @@
         <v>7</v>
       </c>
       <c r="B16" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D16" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F16">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G16" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -904,22 +937,22 @@
         <v>7</v>
       </c>
       <c r="B17" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E17" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F17">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -927,22 +960,22 @@
         <v>7</v>
       </c>
       <c r="B18" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E18" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F18">
         <v>2</v>
       </c>
       <c r="G18" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -950,22 +983,22 @@
         <v>7</v>
       </c>
       <c r="B19" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C19" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D19" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F19">
         <v>2</v>
       </c>
       <c r="G19" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -973,22 +1006,22 @@
         <v>7</v>
       </c>
       <c r="B20" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D20" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="E20" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F20">
         <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -996,22 +1029,22 @@
         <v>7</v>
       </c>
       <c r="B21" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C21" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D21" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E21" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F21">
         <v>2</v>
       </c>
       <c r="G21" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1019,22 +1052,22 @@
         <v>7</v>
       </c>
       <c r="B22" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C22" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D22" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="E22" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F22">
         <v>2</v>
       </c>
       <c r="G22" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1042,22 +1075,22 @@
         <v>7</v>
       </c>
       <c r="B23" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C23" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D23" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="E23" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F23">
         <v>2</v>
       </c>
       <c r="G23" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1065,22 +1098,22 @@
         <v>7</v>
       </c>
       <c r="B24" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D24" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="E24" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F24">
         <v>2</v>
       </c>
       <c r="G24" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1088,22 +1121,22 @@
         <v>7</v>
       </c>
       <c r="B25" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D25" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="E25" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F25">
         <v>2</v>
       </c>
       <c r="G25" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1111,22 +1144,137 @@
         <v>7</v>
       </c>
       <c r="B26" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="E26" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="F26">
         <v>2</v>
       </c>
       <c r="G26" t="s">
-        <v>60</v>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7">
+      <c r="A27" t="s">
+        <v>7</v>
+      </c>
+      <c r="B27" t="s">
+        <v>9</v>
+      </c>
+      <c r="C27" t="s">
+        <v>35</v>
+      </c>
+      <c r="D27" t="s">
+        <v>65</v>
+      </c>
+      <c r="E27" t="s">
+        <v>70</v>
+      </c>
+      <c r="F27">
+        <v>4</v>
+      </c>
+      <c r="G27" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7">
+      <c r="A28" t="s">
+        <v>7</v>
+      </c>
+      <c r="B28" t="s">
+        <v>9</v>
+      </c>
+      <c r="C28" t="s">
+        <v>36</v>
+      </c>
+      <c r="D28" t="s">
+        <v>66</v>
+      </c>
+      <c r="E28" t="s">
+        <v>70</v>
+      </c>
+      <c r="F28">
+        <v>2</v>
+      </c>
+      <c r="G28" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7">
+      <c r="A29" t="s">
+        <v>7</v>
+      </c>
+      <c r="B29" t="s">
+        <v>9</v>
+      </c>
+      <c r="C29" t="s">
+        <v>37</v>
+      </c>
+      <c r="D29" t="s">
+        <v>67</v>
+      </c>
+      <c r="E29" t="s">
+        <v>70</v>
+      </c>
+      <c r="F29">
+        <v>2</v>
+      </c>
+      <c r="G29" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7">
+      <c r="A30" t="s">
+        <v>7</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" t="s">
+        <v>68</v>
+      </c>
+      <c r="E30" t="s">
+        <v>70</v>
+      </c>
+      <c r="F30">
+        <v>2</v>
+      </c>
+      <c r="G30" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7">
+      <c r="A31" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>39</v>
+      </c>
+      <c r="D31" t="s">
+        <v>69</v>
+      </c>
+      <c r="E31" t="s">
+        <v>70</v>
+      </c>
+      <c r="F31">
+        <v>2</v>
+      </c>
+      <c r="G31" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix DZL codes to K111, K104, K204, K107, fix charts render, isolate brand metrics, and add region total row
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -226,10 +226,10 @@
     <t>CL Classic SS Trainer KIDS Black 26</t>
   </si>
   <si>
-    <t>DZL Solitaire</t>
-  </si>
-  <si>
-    <t>🏙️ Same City</t>
+    <t>DZL Redsea</t>
+  </si>
+  <si>
+    <t>🚛 Inter-City</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Isolate shoes from MMS, add brand dropdown in Business tab, enable instant September switch, and restore region total rows
</commit_message>
<xml_diff>
--- a/Reports/Auto_Replenishment_DZL.xlsx
+++ b/Reports/Auto_Replenishment_DZL.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="73">
   <si>
     <t>Brand</t>
   </si>
@@ -227,6 +227,9 @@
   </si>
   <si>
     <t>DZL Redsea</t>
+  </si>
+  <si>
+    <t>🏙️ Same City</t>
   </si>
   <si>
     <t>🚛 Inter-City</t>
@@ -601,7 +604,7 @@
         <v>40</v>
       </c>
       <c r="E2" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F2">
         <v>2</v>
@@ -624,7 +627,7 @@
         <v>41</v>
       </c>
       <c r="E3" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F3">
         <v>6</v>
@@ -647,7 +650,7 @@
         <v>42</v>
       </c>
       <c r="E4" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F4">
         <v>2</v>
@@ -670,7 +673,7 @@
         <v>43</v>
       </c>
       <c r="E5" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F5">
         <v>2</v>
@@ -693,7 +696,7 @@
         <v>44</v>
       </c>
       <c r="E6" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F6">
         <v>2</v>
@@ -716,7 +719,7 @@
         <v>45</v>
       </c>
       <c r="E7" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F7">
         <v>2</v>
@@ -739,7 +742,7 @@
         <v>46</v>
       </c>
       <c r="E8" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F8">
         <v>2</v>
@@ -762,7 +765,7 @@
         <v>47</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F9">
         <v>2</v>
@@ -785,7 +788,7 @@
         <v>48</v>
       </c>
       <c r="E10" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F10">
         <v>2</v>
@@ -808,7 +811,7 @@
         <v>49</v>
       </c>
       <c r="E11" t="s">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="F11">
         <v>2</v>
@@ -837,7 +840,7 @@
         <v>12</v>
       </c>
       <c r="G12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -860,7 +863,7 @@
         <v>4</v>
       </c>
       <c r="G13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -883,7 +886,7 @@
         <v>4</v>
       </c>
       <c r="G14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -906,7 +909,7 @@
         <v>2</v>
       </c>
       <c r="G15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -929,7 +932,7 @@
         <v>4</v>
       </c>
       <c r="G16" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:7">
@@ -952,7 +955,7 @@
         <v>2</v>
       </c>
       <c r="G17" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18" spans="1:7">
@@ -975,7 +978,7 @@
         <v>2</v>
       </c>
       <c r="G18" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19" spans="1:7">
@@ -998,7 +1001,7 @@
         <v>2</v>
       </c>
       <c r="G19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:7">
@@ -1021,7 +1024,7 @@
         <v>2</v>
       </c>
       <c r="G20" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21" spans="1:7">
@@ -1044,7 +1047,7 @@
         <v>2</v>
       </c>
       <c r="G21" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22" spans="1:7">
@@ -1067,7 +1070,7 @@
         <v>2</v>
       </c>
       <c r="G22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23" spans="1:7">
@@ -1090,7 +1093,7 @@
         <v>2</v>
       </c>
       <c r="G23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1113,7 +1116,7 @@
         <v>2</v>
       </c>
       <c r="G24" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="25" spans="1:7">
@@ -1136,7 +1139,7 @@
         <v>2</v>
       </c>
       <c r="G25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1159,7 +1162,7 @@
         <v>2</v>
       </c>
       <c r="G26" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1182,7 +1185,7 @@
         <v>4</v>
       </c>
       <c r="G27" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28" spans="1:7">
@@ -1205,7 +1208,7 @@
         <v>2</v>
       </c>
       <c r="G28" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:7">
@@ -1228,7 +1231,7 @@
         <v>2</v>
       </c>
       <c r="G29" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30" spans="1:7">
@@ -1251,7 +1254,7 @@
         <v>2</v>
       </c>
       <c r="G30" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31" spans="1:7">
@@ -1274,7 +1277,7 @@
         <v>2</v>
       </c>
       <c r="G31" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>